<commit_message>
chore(import): item 1 re-import of the 156 limited-width heading pages, uploaded and previewed; admission-rules spot-check x4, fixes.json entry, report rows
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-campaign.report.xlsx
+++ b/tools/importer/reports/import-campaign.report.xlsx
@@ -58,7 +58,7 @@
     <t>campaign</t>
   </si>
   <si>
-    <t>2026-10-24T06:15:40.361Z</t>
+    <t>2026-10-24T08:03:59.647Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/at/de/100-years</t>
@@ -1840,13 +1840,13 @@
     <t>at/de/onboard-delights.report.json</t>
   </si>
   <si>
-    <t>["hero-campaign","carousel-cards","columns-media","columns-media","columns-media","columns-media"]</t>
+    <t>["profile-tabs","hero-campaign","carousel-cards","columns-media","columns-media","columns-media","columns-media","columns-media"]</t>
   </si>
   <si>
     <t>at/de/onboard-delights</t>
   </si>
   <si>
-    <t>2026-10-24T02:45:36.734Z</t>
+    <t>2026-10-24T06:16:17.650Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/at/de/onboard-delights</t>
@@ -2626,7 +2626,7 @@
     <t>de/de/100-years</t>
   </si>
   <si>
-    <t>2026-10-24T06:15:37.900Z</t>
+    <t>2026-10-24T08:04:15.523Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/de/100-years</t>
@@ -4180,7 +4180,7 @@
     <t>de/de/onboard-delights</t>
   </si>
   <si>
-    <t>2026-10-24T02:58:13.713Z</t>
+    <t>2026-10-24T06:16:14.552Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/de/onboard-delights</t>
@@ -4903,7 +4903,7 @@
     <t>de/en/100-years</t>
   </si>
   <si>
-    <t>2026-10-24T06:15:35.815Z</t>
+    <t>2026-10-24T08:04:33.844Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/100-years</t>
@@ -6403,7 +6403,7 @@
     <t>de/en/onboard-delights</t>
   </si>
   <si>
-    <t>2026-10-24T03:12:07.501Z</t>
+    <t>2026-10-24T06:16:11.748Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/onboard-delights</t>
@@ -7177,7 +7177,7 @@
     <t>gb/en/100-years</t>
   </si>
   <si>
-    <t>2026-10-24T06:15:43.344Z</t>
+    <t>2026-10-24T08:04:48.578Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/gb/en/100-years</t>
@@ -8665,7 +8665,7 @@
     <t>gb/en/onboard-delights</t>
   </si>
   <si>
-    <t>2026-10-24T03:25:07.015Z</t>
+    <t>2026-10-24T06:16:20.392Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/gb/en/onboard-delights</t>
@@ -9496,7 +9496,7 @@
     <t>at/de/100-years/cabin-design</t>
   </si>
   <si>
-    <t>2026-10-24T00:59:53.639Z</t>
+    <t>2026-10-24T08:04:02.602Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/at/de/100-years/cabin-design</t>
@@ -9556,7 +9556,7 @@
     <t>at/de/100-years/destinations</t>
   </si>
   <si>
-    <t>2026-10-24T01:00:05.892Z</t>
+    <t>2026-10-24T08:04:05.799Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/at/de/100-years/destinations</t>
@@ -9571,7 +9571,7 @@
     <t>at/de/100-years/fleet</t>
   </si>
   <si>
-    <t>2026-10-24T01:00:08.824Z</t>
+    <t>2026-10-24T08:04:08.380Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/at/de/100-years/fleet</t>
@@ -9586,7 +9586,7 @@
     <t>at/de/100-years/global-network</t>
   </si>
   <si>
-    <t>2026-10-24T01:00:11.866Z</t>
+    <t>2026-10-24T08:04:11.043Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/at/de/100-years/global-network</t>
@@ -9703,7 +9703,7 @@
     <t>at/de/book-and-manage/stopover</t>
   </si>
   <si>
-    <t>2026-10-24T01:00:19.400Z</t>
+    <t>2026-10-24T08:04:13.652Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/at/de/book-and-manage/stopover</t>
@@ -9925,7 +9925,7 @@
     <t>de/de/100-years/cabin-design</t>
   </si>
   <si>
-    <t>2026-10-24T01:00:38.443Z</t>
+    <t>2026-10-24T08:04:18.962Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/de/100-years/cabin-design</t>
@@ -9973,7 +9973,7 @@
     <t>de/de/100-years/destinations</t>
   </si>
   <si>
-    <t>2026-10-24T01:00:50.191Z</t>
+    <t>2026-10-24T08:04:22.076Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/de/100-years/destinations</t>
@@ -9985,7 +9985,7 @@
     <t>de/de/100-years/fleet</t>
   </si>
   <si>
-    <t>2026-10-24T01:00:53.208Z</t>
+    <t>2026-10-24T08:04:24.506Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/de/100-years/fleet</t>
@@ -9997,7 +9997,7 @@
     <t>de/de/100-years/global-network</t>
   </si>
   <si>
-    <t>2026-10-24T01:00:55.849Z</t>
+    <t>2026-10-24T08:04:27.142Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/de/100-years/global-network</t>
@@ -10096,7 +10096,7 @@
     <t>de/de/book-and-manage/stopover</t>
   </si>
   <si>
-    <t>2026-10-24T01:01:03.164Z</t>
+    <t>2026-10-24T08:04:30.433Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/de/book-and-manage/stopover</t>
@@ -10288,7 +10288,7 @@
     <t>de/en/100-years/cabin-design</t>
   </si>
   <si>
-    <t>2026-10-24T01:01:46.655Z</t>
+    <t>2026-10-24T08:04:35.950Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/100-years/cabin-design</t>
@@ -10339,7 +10339,7 @@
     <t>de/en/100-years/destinations</t>
   </si>
   <si>
-    <t>2026-10-24T01:01:56.642Z</t>
+    <t>2026-10-24T08:04:38.003Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/100-years/destinations</t>
@@ -10351,7 +10351,7 @@
     <t>de/en/100-years/fleet</t>
   </si>
   <si>
-    <t>2026-10-24T01:01:59.093Z</t>
+    <t>2026-10-24T08:04:40.420Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/100-years/fleet</t>
@@ -10363,7 +10363,7 @@
     <t>de/en/100-years/global-network</t>
   </si>
   <si>
-    <t>2026-10-24T01:02:01.370Z</t>
+    <t>2026-10-24T08:04:43.113Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/100-years/global-network</t>
@@ -10459,7 +10459,7 @@
     <t>de/en/book-and-manage/stopover</t>
   </si>
   <si>
-    <t>2026-10-24T01:02:09.701Z</t>
+    <t>2026-10-24T08:04:45.782Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/book-and-manage/stopover</t>
@@ -10654,7 +10654,7 @@
     <t>gb/en/100-years/cabin-design</t>
   </si>
   <si>
-    <t>2026-10-24T01:02:26.932Z</t>
+    <t>2026-10-24T08:04:51.781Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/gb/en/100-years/cabin-design</t>
@@ -10702,7 +10702,7 @@
     <t>gb/en/100-years/destinations</t>
   </si>
   <si>
-    <t>2026-10-24T01:02:37.501Z</t>
+    <t>2026-10-24T08:04:53.817Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/gb/en/100-years/destinations</t>
@@ -10714,7 +10714,7 @@
     <t>gb/en/100-years/fleet</t>
   </si>
   <si>
-    <t>2026-10-24T01:02:39.878Z</t>
+    <t>2026-10-24T08:04:55.807Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/gb/en/100-years/fleet</t>
@@ -10726,7 +10726,7 @@
     <t>gb/en/100-years/global-network</t>
   </si>
   <si>
-    <t>2026-10-24T01:02:42.546Z</t>
+    <t>2026-10-24T08:04:57.893Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/gb/en/100-years/global-network</t>
@@ -10822,7 +10822,7 @@
     <t>gb/en/book-and-manage/stopover</t>
   </si>
   <si>
-    <t>2026-10-24T01:02:50.648Z</t>
+    <t>2026-10-24T08:04:59.922Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/gb/en/book-and-manage/stopover</t>

</xml_diff>